<commit_message>
docs(subsidies): TCO doorgerekend op 100.000 km, EUR 1,70 diesel en 10 cent stroom
Alle drie de invoerwaarden komen nu van Kwekerij Baas zelf. Besparing
EUR 45.989 per truck per jaar, terugverdientijd 5,1 jaar bij middelgroot
(4,6 klein, 5,6 groot).

Toegevoegd: een controle op de haalbaarheid van die 10 cent. Twee trucks
vragen 293.500 kWh per jaar; dat volledig uit eigen opwek halen vraagt om
en nabij 310 kWp aan zonnepanelen die uitsluitend voor de trucks
beschikbaar zijn, plus de accu om dag- en nachtvraag te overbruggen. Komt
de helft van het net, dan loopt de terugverdientijd naar 6,3 jaar.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GWND3AYSABfNFbhavE5Lh7
</commit_message>
<xml_diff>
--- a/docs/subsidies/AanZET TCO-model elektrische trucks.xlsx
+++ b/docs/subsidies/AanZET TCO-model elektrische trucks.xlsx
@@ -592,7 +592,7 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
@@ -697,7 +697,7 @@
         </is>
       </c>
       <c r="C15" s="12" t="n">
-        <v>1.6063</v>
+        <v>1.7</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
@@ -712,7 +712,7 @@
         </is>
       </c>
       <c r="C16" s="13" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="C17" s="12" t="n">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(subsidies): rekenmethode terugverdientijd uitgeschreven, ERS-verbruik in het model
Nieuwe paragraaf 6.7b met de volledige keten van meerprijs naar
terugverdientijd: teller, noemer en uitkomst, met alle tussenstappen.
Toegevoegd een kruiscontrole met contante waarde en interne rentevoet
(18,2 procent over zeven jaar), plus wat de methode negeert.

Het stroomverbruik van de zware trekker in het model staat nu op
1,155 kWh/km uit de Volvo ERS - 1,09 uit de accu plus 6 procent
laadverlies - in plaats van Panteia's 1,4675. De vervanging is op het blad
Panteia-parameters gemarkeerd met de bron. Besparing daarmee 117.863 euro
per jaar en terugverdientijd 3,79 jaar.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GWND3AYSABfNFbhavE5Lh7
</commit_message>
<xml_diff>
--- a/docs/subsidies/AanZET TCO-model elektrische trucks.xlsx
+++ b/docs/subsidies/AanZET TCO-model elektrische trucks.xlsx
@@ -1570,7 +1570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:J48"/>
+  <dimension ref="B1:K48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1583,6 +1583,7 @@
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="90" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1803,7 +1804,7 @@
         <v>0.3413502921361025</v>
       </c>
       <c r="D10" s="32" t="n">
-        <v>1.4675</v>
+        <v>1.155</v>
       </c>
       <c r="E10" s="33" t="n">
         <v>0.09164053028160001</v>
@@ -1823,6 +1824,11 @@
       <c r="J10" s="30" t="inlineStr">
         <is>
           <t>N3 Trekker</t>
+        </is>
+      </c>
+      <c r="K10" s="27" t="inlineStr">
+        <is>
+          <t>VERVANGEN — Volvo ERS 18-08-2026, route Ens-Naaldwijk: 1,09 kWh/km uit de accu + 6% laadverlies</t>
         </is>
       </c>
     </row>

</xml_diff>